<commit_message>
Added saving screenshots to /:C when human = detected, update PyTorch environment to support CUDA and enable GPU execution
</commit_message>
<xml_diff>
--- a/db/logs_detection_ur3.xlsx
+++ b/db/logs_detection_ur3.xlsx
@@ -2,28 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="datalogs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -51,7 +57,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -59,9 +65,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -424,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:N113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -438,78 +447,78 @@
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="29" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="12" max="13"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>id_detection</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>id_camera</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>ai_model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>hardware_setup</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>detection_start_time</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>detection_end_time</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>duration_s</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>average_fps</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>average_model_accuracy</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>average_inference_time_ms</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>tcp_x</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>tcp_y</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>tcp_z</t>
         </is>
@@ -5966,6 +5975,600 @@
         <v>0</v>
       </c>
       <c r="N102" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:29</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:42</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="I103" s="2" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="J103" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K103" s="2" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="L103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N103" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:44</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:44</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I104" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="J104" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K104" s="2" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="L104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N104" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:44</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:44</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I105" s="2" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="J105" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K105" s="2" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="L105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N105" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:06:46</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:13</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="n">
+        <v>27.56</v>
+      </c>
+      <c r="I106" s="2" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="J106" s="2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="L106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N106" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:17</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:27</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>9.77</v>
+      </c>
+      <c r="I107" s="2" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N107" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:32</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:45</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>13.51</v>
+      </c>
+      <c r="I108" s="2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:48</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:53</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="I109" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="J109" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="L109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:07:55</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:08:04</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="I110" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="J110" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K110" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="L110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:23</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:32</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="I111" s="2" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="J111" s="2" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="L111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:33</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:35</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="I112" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N112" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:37</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14 22:17:39</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="I113" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J113" s="2" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K113" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="L113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N113" s="2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added logger to mySQL to transfer data of detections in real time data exchange
</commit_message>
<xml_diff>
--- a/db/logs_detection_ur3.xlsx
+++ b/db/logs_detection_ur3.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N113"/>
+  <dimension ref="A1:N147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6572,6 +6572,1842 @@
         <v>0</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:49</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:49</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I114" s="2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="J114" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N114" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:49</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:49</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N115" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:52</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:52</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I116" s="2" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N116" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:52</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:52</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I117" s="2" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K117" s="2" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N117" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:53</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:41:53</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I118" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J118" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K118" s="2" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="L118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N118" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:04</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:06</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="I119" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J119" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K119" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N119" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:09</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:11</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="I120" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K120" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L120" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:14</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:17</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="I121" s="2" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J121" s="2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K121" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="L121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N121" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:18</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:21</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="I122" s="2" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="J122" s="2" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="K122" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="L122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N122" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:22</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:25</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I123" s="2" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="J123" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K123" s="2" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="L123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N123" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:27</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:30</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="I124" s="2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="J124" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K124" s="2" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="L124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:31</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:37</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="J125" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:39</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:42:39</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:08</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:11</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:13</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:16</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J128" s="2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K128" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:18</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:20</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="I129" s="2" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="J129" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K129" s="2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="L129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:22</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:25</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="I130" s="2" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="J130" s="2" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="K130" s="2" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="L130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N130" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:27</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:29</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="I131" s="2" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="J131" s="2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="K131" s="2" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="L131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N131" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:31</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:36</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="I132" s="2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="J132" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K132" s="2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="L132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N132" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:38</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:38</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I133" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J133" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K133" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="L133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N133" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:38</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:38</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I134" s="2" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="J134" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="K134" s="2" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="L134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N134" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:39</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:39</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I135" s="2" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="J135" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="K135" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="L135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N135" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:58</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:58</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I136" s="2" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="J136" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="K136" s="2" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="L136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N136" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:54:58</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:55:02</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="I137" s="2" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="J137" s="2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K137" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="L137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N137" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:55:04</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:55:04</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I138" s="2" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="J138" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K138" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="L138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N138" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:18</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:18</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I139" s="2" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="J139" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="K139" s="2" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="L139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N139" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:18</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:18</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="I140" s="2" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J140" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K140" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="L140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N140" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:19</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:19</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I141" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J141" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K141" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N141" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:20</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:20</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="J142" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K142" s="2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="L142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N142" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:22</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:22</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="J143" s="2" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="K143" s="2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="L143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N143" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:23</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:23</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I144" s="2" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J144" s="2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="K144" s="2" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="L144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N144" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:24</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:25</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I145" s="2" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="J145" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K145" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="L145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N145" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:26</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:27</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="J146" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K146" s="2" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="L146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N146" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>requires checking</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>yolov8n-pose.pt</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>no cobot</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:28</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16 10:58:28</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="I147" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="J147" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="K147" s="2" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="L147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N147" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>